<commit_message>
Data TAble Sorting Validation Commite
</commit_message>
<xml_diff>
--- a/Data/Activity Dashboard/Group Widgets/Top Application/TopApplication.xlsx
+++ b/Data/Activity Dashboard/Group Widgets/Top Application/TopApplication.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>exportType</t>
   </si>
@@ -36,6 +36,12 @@
   </si>
   <si>
     <t>isDataValion</t>
+  </si>
+  <si>
+    <t>isTableSorting</t>
+  </si>
+  <si>
+    <t>isTSValidation</t>
   </si>
   <si>
     <t>excel</t>
@@ -985,9 +991,10 @@
   <cols>
     <col min="1" max="1" width="30.2857142857143" customWidth="1"/>
     <col min="2" max="2" width="29.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="10.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -997,18 +1004,29 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="C2" t="b">
+      <c r="E2" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="E2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>